<commit_message>
Add Classic Pickled Carrots SOP, Golden Hour and Harvest Bowl recipe cards
New documents added and organized into folder structure:
- Classic Quick Pickled Carrots SOP v1 (Miscellaneous) — foundational
  pickled carrot with 60-day shelf life and 5 approved variations
- Golden Hour Recipe Card v1 — Mediterranean bowl with lemon-herb
  chicken and roasted sweet potato (5-unit batch)
- Harvest Bowl Recipe Card v1 — Southern comfort bowl with whipped
  sweet potato and smoked chicken (5-unit batch)

Master recipe database updated: 26 recipes, 3 SOPs complete,
3 recipe cards complete.

https://claude.ai/code/session_01RoU8RfG3RfKf7Zo4boqHgn
</commit_message>
<xml_diff>
--- a/Recipes/CC_Master_Recipe_Database_v1.xlsx
+++ b/Recipes/CC_Master_Recipe_Database_v1.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -548,7 +548,6 @@
           <t>Recipes/Miscellaneous/Asian_Ginger_Pickled_Carrots_SOP_v1.docx</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>30 days</t>
@@ -683,8 +682,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -710,7 +707,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>Weekly staple</t>
@@ -743,8 +739,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -770,7 +764,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>Weekly staple</t>
@@ -803,8 +796,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -830,7 +821,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>Weekly staple</t>
@@ -863,8 +853,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -890,7 +878,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>Surplus hash browns</t>
@@ -923,8 +910,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>2 days</t>
@@ -950,7 +935,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>Varies by surplus produce</t>
@@ -983,8 +967,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1010,8 +992,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1039,8 +1019,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1066,8 +1044,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1095,8 +1071,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1122,7 +1096,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>Surplus sweet potatoes</t>
@@ -1155,8 +1128,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1182,8 +1153,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1211,8 +1180,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1238,8 +1205,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1267,8 +1232,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>5 days</t>
@@ -1294,7 +1257,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>Surplus broccoli</t>
@@ -1324,14 +1286,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/GoldenHour_RecipeCard_v1.docx</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>5 days</t>
+          <t>3-4 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1341,7 +1306,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Dairy (feta)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1354,10 +1319,9 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Surplus sweet potatoes; from Week 11</t>
+          <t>Mediterranean bowl; lemon-herb chicken + roasted sweet potato</t>
         </is>
       </c>
     </row>
@@ -1384,14 +1348,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/HarvestBowl_RecipeCard_v1.docx</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>5 days</t>
+          <t>3-4 days</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1401,7 +1368,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Dairy (butter, cream), Gluten (cornbread crumble)</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1414,10 +1381,9 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Surplus sweet potatoes; from Week 11</t>
+          <t>Southern comfort bowl; whipped sweet potato + smoked chicken</t>
         </is>
       </c>
     </row>
@@ -1447,8 +1413,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>5 days</t>
@@ -1474,8 +1438,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1503,8 +1465,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>5 days</t>
@@ -1530,8 +1490,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1559,8 +1517,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>5 days</t>
@@ -1586,8 +1542,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1615,8 +1569,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1642,8 +1594,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1671,8 +1621,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1698,7 +1646,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>Surplus sweet potatoes</t>
@@ -1731,8 +1678,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1758,7 +1703,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>Week 11; surplus strawberries</t>
@@ -1791,8 +1735,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1818,7 +1760,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>Week 11; surplus brisket</t>
@@ -1851,8 +1792,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>5 days</t>
@@ -1878,7 +1817,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>Week 11; surplus brisket</t>
@@ -1911,8 +1849,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>5 days</t>
@@ -1938,7 +1874,6 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>Week 11</t>
@@ -1971,8 +1906,6 @@
           <t>Needed</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>3 days</t>
@@ -1998,10 +1931,77 @@
           <t>03/15/2026</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>Week 11; surplus strawberries</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RCP-026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Classic Quick Pickled Carrots</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Recipes/Miscellaneous/Classic_Quick_Pickled_Carrots_SOP_v1.docx</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>60 days</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>02/15/2026</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Foundational pickled carrot; 5 approved variations</t>
         </is>
       </c>
     </row>
@@ -2092,8 +2092,6 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2126,8 +2124,6 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2160,8 +2156,6 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2194,8 +2188,6 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2228,8 +2220,6 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2262,8 +2252,6 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2296,14 +2284,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2326,14 +2311,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2356,14 +2338,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2386,14 +2365,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2416,14 +2392,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2446,14 +2419,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2476,14 +2446,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2506,14 +2473,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2536,14 +2500,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2566,14 +2527,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2596,14 +2554,11 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2729,16 +2684,16 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
         <v>3</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -2767,13 +2722,13 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>21</v>

</xml_diff>

<commit_message>
Add 9 new recipes: SOPs and recipe cards organized into database
New SOPs (3):
- BBQ Chicken Wrap (Wraps/) — oven-smoked pulled chicken, 2-day production
- Turkey Club Wrap (Wraps/)
- Smoked Chicken Salad (Salads/) — 75-serving catering scale

New Recipe Cards (6):
- Strawberry Fields Salad — romaine, goat cheese, candied pecans
- The Heights Bowl — Asian grain bowl, sweet potato noodles
- The Plant Power Bowl — VEGAN, quinoa/rice, black beans, chickpeas
- The Revival Bowl — Mediterranean, harissa/tzatziki/hummus
- The Rooted Bowl — ancient grain blend, broccoli pesto
- The Common Table Bowl — Brussels, apples, goat cheese

Master database now: 32 recipes, 8 SOPs complete, 10 recipe cards complete.

https://claude.ai/code/session_01RoU8RfG3RfKf7Zo4boqHgn
</commit_message>
<xml_diff>
--- a/Recipes/CC_Master_Recipe_Database_v1.xlsx
+++ b/Recipes/CC_Master_Recipe_Database_v1.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1680,12 +1680,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Needed</t>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/Strawberry_Fields_Salad_RecipeCard_v1.docx</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>3 days</t>
+          <t>3-4 days</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1695,7 +1700,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Milk (goat cheese), Tree Nuts (pecans), Mustard</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1710,7 +1715,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Week 11; surplus strawberries</t>
+          <t>Romaine, strawberries, goat cheese, candied pecans, balsamic vinaigrette</t>
         </is>
       </c>
     </row>
@@ -2063,6 +2068,618 @@
       <c r="N28" t="inlineStr">
         <is>
           <t>New Caney only; 3 units Monday PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RCP-028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>BBQ Chicken Wrap</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Wraps</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Recipes/Wraps/BBQ_Chicken_Wrap_SOP_v1.md</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>3-5 days</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Dairy (pepperjack), Gluten (tortilla)</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Oven-smoked pulled chicken, KC BBQ sauce, coleslaw, pepperjack</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>RCP-029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Turkey Club Wrap</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Wraps</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Recipes/Wraps/Turkey_Club_Wrap_SOP_v1.md</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>3-5 days</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Dairy, Gluten, Eggs (mayo)</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Turkey, bacon, Swiss, lettuce, tomato</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>RCP-030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Smoked Chicken Salad</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Salads</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Recipes/Salads/Smoked_Chicken_Salad_SOP_v1.docx</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>3 days</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Eggs (mayo), Tree Nuts (pecans)</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>BBQ-boosted; crispy shallots, toasted pecans, pickled red onion; 75-serving catering scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>RCP-031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Strawberry Fields Salad</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Salads</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/Strawberry_Fields_Salad_RecipeCard_v1.docx</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>3-4 days</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Milk (goat cheese), Tree Nuts (pecans), Mustard</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Romaine, strawberries, goat cheese, candied pecans, balsamic vinaigrette</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>RCP-032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>The Heights Bowl</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Bowls</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/Heights_Bowl_RecipeCard_v1.txt</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>4 days</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Tree Nuts (almonds, cashews), Soy, Fish (fish sauce)</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Asian grain bowl; sweet potato noodles or rice, grilled chicken/tofu, bok choy, shiitake</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>RCP-033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>The Plant Power Bowl</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Bowls</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/Plant_Power_Bowl_RecipeCard_v1.txt</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>5 days</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Sesame (tahini)</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>VEGAN; quinoa/rice, black beans, roasted chickpeas, sweet potato, Brussels, tahini-lemon dressing</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>RCP-034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>The Revival Bowl</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Bowls</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/Revival_Bowl_RecipeCard_v1.txt</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>5 days</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Milk (mozzarella, tzatziki), Sesame (hummus)</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Mediterranean; basmati rice, grilled chicken, summer squash, roasted broccoli, harissa/tzatziki/hummus</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>RCP-035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>The Rooted Bowl</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Bowls</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/Rooted_Bowl_RecipeCard_v1.txt</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>5 days</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Gluten (farro), Soy (miso)</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Ancient grain blend (quinoa/farro/wild rice), herb-roasted chicken, sweet potato, broccoli pesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>RCP-036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>The Common Table Bowl</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Bowls</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Recipes/RecipeCards/Common_Table_Bowl_RecipeCard_v1.txt</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>5 days</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Milk (goat cheese), Tree Nuts (pecans/almonds)</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>01/2026</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Brown rice/quinoa, herb-roasted chicken, Brussels, apples, goat cheese, honey-white balsamic</t>
         </is>
       </c>
     </row>
@@ -2688,16 +3305,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -2707,10 +3324,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -2726,16 +3343,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -2783,16 +3400,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>